<commit_message>
update raw data files from atlas.ti
</commit_message>
<xml_diff>
--- a/codes_catalog.xlsx
+++ b/codes_catalog.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="159">
   <si>
     <t>name</t>
   </si>
@@ -97,7 +97,7 @@
     <t>Lack of trust in programming transformation tools</t>
   </si>
   <si>
-    <t>Selective, Risk-Aware, and Human-Controlled Use of Tool Support</t>
+    <t>Tooling Constraints and Control Mechanisms</t>
   </si>
   <si>
     <t>Difficulty in following language evolution</t>
@@ -193,6 +193,9 @@
     <t>Reliance on static analysis to detect SCR opportunities</t>
   </si>
   <si>
+    <t>Selective and Human-Controlled Use of Tool Support</t>
+  </si>
+  <si>
     <t>Framework/library dependencies hinder SCR efforts</t>
   </si>
   <si>
@@ -352,7 +355,7 @@
     <t>Disabling warnings to keep systems compiling</t>
   </si>
   <si>
-    <t>Technical Constraints</t>
+    <t>Managing Technical Constraints and Compatibility</t>
   </si>
   <si>
     <t>Programming language complexity might hinder SCR efforts</t>
@@ -1359,26 +1362,20 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="20" t="s">
         <v>52</v>
       </c>
       <c r="B30" t="s">
         <v>4</v>
       </c>
-      <c r="C30" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B31" t="s">
         <v>4</v>
-      </c>
-      <c r="C31" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -1422,23 +1419,23 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B36" t="s">
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="22" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B37" t="s">
         <v>4</v>
@@ -1449,7 +1446,7 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="23" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B38" t="s">
         <v>4</v>
@@ -1458,20 +1455,17 @@
         <v>40</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="24" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
-      </c>
-      <c r="C39" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B40" t="s">
         <v>4</v>
@@ -1479,73 +1473,73 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B41" t="s">
         <v>4</v>
       </c>
       <c r="C41" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="26" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B42" t="s">
         <v>4</v>
       </c>
       <c r="C42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="27" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B43" t="s">
         <v>4</v>
       </c>
       <c r="C43" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B44" t="s">
         <v>4</v>
       </c>
       <c r="C44" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B45" t="s">
         <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B46" t="s">
         <v>4</v>
       </c>
       <c r="C46" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="28" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B47" t="s">
         <v>4</v>
@@ -1553,26 +1547,23 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B48" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B49" t="s">
         <v>4</v>
-      </c>
-      <c r="C49" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="27" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B50" t="s">
         <v>4</v>
@@ -1580,29 +1571,29 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="27" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B51" t="s">
         <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="22" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B52" t="s">
         <v>4</v>
       </c>
       <c r="C52" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="29" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B53" t="s">
         <v>4</v>
@@ -1613,7 +1604,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B54" t="s">
         <v>4</v>
@@ -1624,18 +1615,18 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B55" t="s">
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="30" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B56" t="s">
         <v>4</v>
@@ -1646,18 +1637,18 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B57" t="s">
         <v>4</v>
       </c>
       <c r="C57" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B58" t="s">
         <v>4</v>
@@ -1665,7 +1656,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="26" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B59" t="s">
         <v>4</v>
@@ -1676,7 +1667,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B60" t="s">
         <v>4</v>
@@ -1687,7 +1678,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="31" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B61" t="s">
         <v>4</v>
@@ -1695,7 +1686,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B62" t="s">
         <v>4</v>
@@ -1703,7 +1694,7 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="21" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B63" t="s">
         <v>4</v>
@@ -1714,7 +1705,7 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B64" t="s">
         <v>4</v>
@@ -1725,7 +1716,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B65" t="s">
         <v>4</v>
@@ -1733,21 +1724,21 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="32" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B66" t="s">
         <v>4</v>
       </c>
       <c r="C66" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B67" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C67" t="s">
         <v>19</v>
@@ -1755,18 +1746,18 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="33" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B68" t="s">
         <v>4</v>
       </c>
       <c r="C68" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B69" t="s">
         <v>4</v>
@@ -1777,18 +1768,18 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B70" t="s">
         <v>4</v>
       </c>
       <c r="C70" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B71" t="s">
         <v>4</v>
@@ -1799,7 +1790,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B72" t="s">
         <v>4</v>
@@ -1807,18 +1798,18 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="34" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B73" t="s">
         <v>4</v>
       </c>
       <c r="C73" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B74" t="s">
         <v>4</v>
@@ -1829,7 +1820,7 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="27" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B75" t="s">
         <v>4</v>
@@ -1837,7 +1828,7 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B76" t="s">
         <v>4</v>
@@ -1848,7 +1839,7 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="35" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B77" t="s">
         <v>4</v>
@@ -1859,18 +1850,18 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B78" t="s">
         <v>4</v>
       </c>
       <c r="C78" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="31" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B79" t="s">
         <v>4</v>
@@ -1881,7 +1872,7 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="36" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B80" t="s">
         <v>4</v>
@@ -1890,42 +1881,33 @@
         <v>24</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B81" t="s">
         <v>4</v>
       </c>
-      <c r="C81" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B82" t="s">
         <v>4</v>
       </c>
-      <c r="C82" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B83" t="s">
         <v>4</v>
-      </c>
-      <c r="C83" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="30" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B84" t="s">
         <v>4</v>
@@ -1933,7 +1915,7 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B85" t="s">
         <v>4</v>
@@ -1944,7 +1926,7 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B86" t="s">
         <v>4</v>
@@ -1952,18 +1934,18 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B87" t="s">
         <v>4</v>
       </c>
       <c r="C87" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B88" t="s">
         <v>4</v>
@@ -1974,7 +1956,7 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B89" t="s">
         <v>4</v>
@@ -1983,42 +1965,33 @@
         <v>30</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B90" t="s">
         <v>4</v>
       </c>
-      <c r="C90" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="19" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B91" t="s">
         <v>4</v>
       </c>
-      <c r="C91" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="22" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B92" t="s">
         <v>4</v>
-      </c>
-      <c r="C92" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B93" t="s">
         <v>4</v>
@@ -2026,7 +1999,7 @@
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B94" t="s">
         <v>4</v>
@@ -2037,7 +2010,7 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B95" t="s">
         <v>4</v>
@@ -2048,7 +2021,7 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="15" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B96" t="s">
         <v>4</v>
@@ -2056,15 +2029,15 @@
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B97" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B98" t="s">
         <v>4</v>
@@ -2072,7 +2045,7 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B99" t="s">
         <v>4</v>
@@ -2080,7 +2053,7 @@
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="24" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B100" t="s">
         <v>4</v>
@@ -2088,7 +2061,7 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" s="26" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B101" t="s">
         <v>4</v>
@@ -2096,7 +2069,7 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B102" t="s">
         <v>4</v>
@@ -2104,7 +2077,7 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" s="33" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B103" t="s">
         <v>4</v>
@@ -2112,7 +2085,7 @@
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" s="33" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B104" t="s">
         <v>4</v>
@@ -2120,7 +2093,7 @@
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" s="34" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B105" t="s">
         <v>4</v>
@@ -2128,7 +2101,7 @@
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" s="22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B106" t="s">
         <v>4</v>
@@ -2136,7 +2109,7 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B107" t="s">
         <v>4</v>
@@ -2144,7 +2117,7 @@
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" s="21" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B108" t="s">
         <v>4</v>
@@ -2152,18 +2125,18 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B109" t="s">
         <v>4</v>
       </c>
       <c r="C109" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" s="34" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B110" t="s">
         <v>4</v>
@@ -2171,18 +2144,18 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B111" t="s">
         <v>4</v>
       </c>
       <c r="C111" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B112" t="s">
         <v>4</v>
@@ -2190,40 +2163,40 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="9" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B113" t="s">
         <v>4</v>
       </c>
       <c r="C113" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B114" t="s">
         <v>4</v>
       </c>
       <c r="C114" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B115" t="s">
         <v>4</v>
       </c>
       <c r="C115" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B116" t="s">
         <v>4</v>
@@ -2231,13 +2204,13 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B117" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C117" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>